<commit_message>
Refine SOC accounting logic to incorporate transition periods and improve CSV data consistency.
</commit_message>
<xml_diff>
--- a/data/my_project/raw/my_data.xlsx
+++ b/data/my_project/raw/my_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tboll\DELL_local_code\CarbonIQ\agricultural-land-management\data\my_project\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9474F7B-5606-4A0F-A570-6F4EBDC95826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560D2A48-5A4E-404C-90A8-AA9FA17F7EDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28845" yWindow="1545" windowWidth="28770" windowHeight="12645" activeTab="6" xr2:uid="{9B51F04F-7C9B-484C-9CA7-D1EDE120DFB6}"/>
+    <workbookView xWindow="750" yWindow="1245" windowWidth="26400" windowHeight="15645" firstSheet="1" activeTab="7" xr2:uid="{9B51F04F-7C9B-484C-9CA7-D1EDE120DFB6}"/>
   </bookViews>
   <sheets>
     <sheet name="projects" sheetId="5" r:id="rId1"/>
@@ -20,8 +20,10 @@
     <sheet name="soc_samples" sheetId="1" r:id="rId5"/>
     <sheet name="soc_stock_change_factors" sheetId="7" r:id="rId6"/>
     <sheet name="strata" sheetId="3" r:id="rId7"/>
+    <sheet name="calc" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="223">
   <si>
     <t>sample_id</t>
   </si>
@@ -416,9 +418,6 @@
     <t>IPCC_default_demo</t>
   </si>
   <si>
-    <t>v1</t>
-  </si>
-  <si>
     <t>illustrative</t>
   </si>
   <si>
@@ -654,6 +653,66 @@
   </si>
   <si>
     <t>Project subsoil; early signs of SOC stabilization under improved management.</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
+    <t>NSW_DPI_DPIRD_synthesis</t>
+  </si>
+  <si>
+    <t>v1.0</t>
+  </si>
+  <si>
+    <t>Baseline typical; conservative multipliers for sandy loam Tenosols; uncertainty ±20%.</t>
+  </si>
+  <si>
+    <t>Improved grazing (rest periods, modest pasture improvement); uncertainty ±15%.</t>
+  </si>
+  <si>
+    <t>Rotational grazing with multi‑paddock rest; apply only when documented rest periods and groundcover targets met; uncertainty ±15%.</t>
+  </si>
+  <si>
+    <t>medium_high_input</t>
+  </si>
+  <si>
+    <t>irrigated_seasonal</t>
+  </si>
+  <si>
+    <t>USDA regional syntheses</t>
+  </si>
+  <si>
+    <t>full inversion tillage with low residue retention reduces surface SOC and accelerates decomposition; apply conservative bounds (multiplier_low ≈ 0.75, multiplier_high ≈ 0.95). Ramp effect over 5 years to reflect gradual SOC decline under continued practice. Evidence: national/regional CSA reviews and tillage meta‑analyses.</t>
+  </si>
+  <si>
+    <t>USDA / peer literature</t>
+  </si>
+  <si>
+    <t>typical conventional tillage; moderate SOC loss risk relative to reduced‑till. Use lower bound for crediting; multiplier bounds ≈ 0.82–1.05. Ramp 5 years.</t>
+  </si>
+  <si>
+    <t>UC Davis / peer studies</t>
+  </si>
+  <si>
+    <t>reduced till combined with cover cropping can increase net ecosystem C balance, but effectiveness is site‑specific (soil texture, cover crop species, biomass). Use monitoring triggers (documented cover crop biomass, residue retention) before applying full multipliers; multiplier bounds ≈ 0.95–1.30. Ramp 7 years to reflect slower SOC accrual and interannual variability. Recent California studies show cover crop + reduced till benefits depend strongly on texture and local conditions.</t>
+  </si>
+  <si>
+    <t>soc_impact</t>
+  </si>
+  <si>
+    <t>moderate_impact</t>
+  </si>
+  <si>
+    <t>low_impact</t>
+  </si>
+  <si>
+    <t>slow_impact</t>
+  </si>
+  <si>
+    <t>transition_period_years</t>
+  </si>
+  <si>
+    <t>stock_tC_ha</t>
   </si>
 </sst>
 </file>
@@ -661,9 +720,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -679,13 +738,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -700,12 +772,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1067,7 +1146,7 @@
         <v>102</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>103</v>
@@ -1082,7 +1161,7 @@
         <v>106</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>107</v>
@@ -1114,7 +1193,7 @@
         <v>114</v>
       </c>
       <c r="C2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D2" t="s">
         <v>115</v>
@@ -1155,19 +1234,19 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B3" t="s">
         <v>142</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D3" t="s">
         <v>143</v>
       </c>
-      <c r="C3" t="s">
-        <v>141</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>144</v>
-      </c>
-      <c r="E3" t="s">
-        <v>145</v>
       </c>
       <c r="F3" t="s">
         <v>117</v>
@@ -1194,7 +1273,7 @@
         <v>150.5</v>
       </c>
       <c r="N3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O3" t="s">
         <v>118</v>
@@ -1249,7 +1328,7 @@
         <v>37</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>62</v>
@@ -1320,13 +1399,13 @@
         <v>49</v>
       </c>
       <c r="E2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F2" t="s">
         <v>146</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>147</v>
-      </c>
-      <c r="G2" t="s">
-        <v>148</v>
       </c>
       <c r="H2" t="s">
         <v>93</v>
@@ -1391,13 +1470,13 @@
         <v>49</v>
       </c>
       <c r="E3" t="s">
+        <v>145</v>
+      </c>
+      <c r="F3" t="s">
         <v>146</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>147</v>
-      </c>
-      <c r="G3" t="s">
-        <v>148</v>
       </c>
       <c r="H3" t="s">
         <v>97</v>
@@ -1462,13 +1541,13 @@
         <v>49</v>
       </c>
       <c r="E4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F4" t="s">
         <v>146</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>147</v>
-      </c>
-      <c r="G4" t="s">
-        <v>148</v>
       </c>
       <c r="H4" t="s">
         <v>99</v>
@@ -1521,7 +1600,7 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -1530,25 +1609,25 @@
         <v>2024</v>
       </c>
       <c r="D5" t="s">
+        <v>132</v>
+      </c>
+      <c r="E5" t="s">
         <v>133</v>
       </c>
-      <c r="E5" t="s">
-        <v>134</v>
-      </c>
       <c r="F5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I5" t="b">
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K5" t="s">
         <v>98</v>
@@ -1572,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="R5" t="s">
+        <v>155</v>
+      </c>
+      <c r="S5" t="s">
         <v>156</v>
-      </c>
-      <c r="S5" t="s">
-        <v>157</v>
       </c>
       <c r="T5">
         <v>1.25</v>
@@ -1653,7 +1732,7 @@
         <v>32</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>33</v>
@@ -1721,7 +1800,7 @@
         <v>175</v>
       </c>
       <c r="J2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K2" t="s">
         <v>45</v>
@@ -1786,7 +1865,7 @@
         <v>210</v>
       </c>
       <c r="J3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K3" t="s">
         <v>54</v>
@@ -1824,16 +1903,16 @@
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C4" t="s">
         <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E4" s="3">
         <v>-31.5</v>
@@ -1851,31 +1930,31 @@
         <v>135</v>
       </c>
       <c r="J4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="L4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M4" t="s">
         <v>47</v>
       </c>
       <c r="N4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
       </c>
       <c r="R4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="S4" t="b">
         <v>0</v>
@@ -1887,21 +1966,21 @@
         <v>58</v>
       </c>
       <c r="V4" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E5" s="3">
         <v>-31.502500000000001</v>
@@ -1919,31 +1998,31 @@
         <v>190</v>
       </c>
       <c r="J5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="L5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M5" t="s">
         <v>47</v>
       </c>
       <c r="N5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
       </c>
       <c r="R5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="S5" t="b">
         <v>0</v>
@@ -1955,21 +2034,21 @@
         <v>58</v>
       </c>
       <c r="V5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E6" s="3">
         <v>-31.498000000000001</v>
@@ -1987,31 +2066,31 @@
         <v>80</v>
       </c>
       <c r="J6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K6" t="s">
+        <v>185</v>
+      </c>
+      <c r="L6" t="s">
         <v>186</v>
-      </c>
-      <c r="L6" t="s">
-        <v>187</v>
       </c>
       <c r="M6" t="s">
         <v>47</v>
       </c>
       <c r="N6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
       </c>
       <c r="R6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="S6" t="b">
         <v>0</v>
@@ -2023,7 +2102,7 @@
         <v>52</v>
       </c>
       <c r="V6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -2085,10 +2164,10 @@
         <v>123</v>
       </c>
       <c r="F2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -2108,15 +2187,15 @@
         <v>123</v>
       </c>
       <c r="F3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B4" t="s">
         <v>70</v>
@@ -2131,18 +2210,18 @@
         <v>123</v>
       </c>
       <c r="F4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C5">
         <v>30</v>
@@ -2151,13 +2230,13 @@
         <v>48</v>
       </c>
       <c r="E5" t="s">
+        <v>165</v>
+      </c>
+      <c r="F5" t="s">
         <v>166</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>167</v>
-      </c>
-      <c r="G5" t="s">
-        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -2252,7 +2331,7 @@
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B2" t="s">
         <v>19</v>
@@ -2308,7 +2387,7 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
@@ -2364,7 +2443,7 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B4" t="s">
         <v>19</v>
@@ -2420,19 +2499,19 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F5" s="1">
         <v>45181</v>
@@ -2459,7 +2538,7 @@
         <v>5.9</v>
       </c>
       <c r="N5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="O5" t="s">
         <v>24</v>
@@ -2474,24 +2553,24 @@
         <v>25</v>
       </c>
       <c r="S5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F6" s="1">
         <v>45181</v>
@@ -2518,7 +2597,7 @@
         <v>6</v>
       </c>
       <c r="N6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="O6" t="s">
         <v>24</v>
@@ -2533,24 +2612,24 @@
         <v>25</v>
       </c>
       <c r="S6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F7" s="1">
         <v>45182</v>
@@ -2577,7 +2656,7 @@
         <v>5.8</v>
       </c>
       <c r="N7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="O7" t="s">
         <v>24</v>
@@ -2592,24 +2671,24 @@
         <v>25</v>
       </c>
       <c r="S7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F8" s="1">
         <v>45182</v>
@@ -2636,7 +2715,7 @@
         <v>5.9</v>
       </c>
       <c r="N8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="O8" t="s">
         <v>24</v>
@@ -2651,21 +2730,21 @@
         <v>25</v>
       </c>
       <c r="S8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E9" t="s">
         <v>22</v>
@@ -2695,7 +2774,7 @@
         <v>6.2</v>
       </c>
       <c r="N9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="O9" t="s">
         <v>24</v>
@@ -2710,21 +2789,21 @@
         <v>25</v>
       </c>
       <c r="S9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C10" t="s">
         <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E10" t="s">
         <v>22</v>
@@ -2754,7 +2833,7 @@
         <v>6.1</v>
       </c>
       <c r="N10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="O10" t="s">
         <v>24</v>
@@ -2769,7 +2848,7 @@
         <v>25</v>
       </c>
       <c r="S10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -2779,198 +2858,496 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6806E13-BA06-4F43-9BFB-FE354E4A58FA}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B2" t="s">
         <v>49</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>57</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>71</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>76</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>0.8</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2" t="s">
+        <v>129</v>
+      </c>
+      <c r="J2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3">
+        <v>0.8</v>
+      </c>
+      <c r="G3">
+        <v>1.08</v>
+      </c>
+      <c r="H3">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="I3" t="s">
+        <v>129</v>
+      </c>
+      <c r="J3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" t="s">
         <v>130</v>
       </c>
-      <c r="I2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="D4" t="s">
+        <v>131</v>
+      </c>
+      <c r="E4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4">
+        <v>0.8</v>
+      </c>
+      <c r="G4">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="H4">
+        <v>1.2</v>
+      </c>
+      <c r="I4" t="s">
+        <v>129</v>
+      </c>
+      <c r="J4" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>203</v>
+      </c>
+      <c r="B5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H5">
+        <v>1.05</v>
+      </c>
+      <c r="I5" t="s">
+        <v>129</v>
+      </c>
+      <c r="J5" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>203</v>
+      </c>
+      <c r="B6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F6">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="G6">
+        <v>1.08</v>
+      </c>
+      <c r="H6">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="I6" t="s">
+        <v>136</v>
+      </c>
+      <c r="J6" t="s">
+        <v>205</v>
+      </c>
+      <c r="K6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="D7" t="s">
+        <v>160</v>
+      </c>
+      <c r="E7" t="s">
+        <v>147</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="H7">
+        <v>1.08</v>
+      </c>
+      <c r="I7" t="s">
+        <v>204</v>
+      </c>
+      <c r="J7" t="s">
+        <v>205</v>
+      </c>
+      <c r="K7" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B8" t="s">
+        <v>132</v>
+      </c>
+      <c r="C8" t="s">
+        <v>162</v>
+      </c>
+      <c r="D8" t="s">
+        <v>160</v>
+      </c>
+      <c r="E8" t="s">
+        <v>147</v>
+      </c>
+      <c r="F8">
+        <v>0.95</v>
+      </c>
+      <c r="G8">
+        <v>0.95</v>
+      </c>
+      <c r="H8">
+        <v>0.98</v>
+      </c>
+      <c r="I8" t="s">
+        <v>204</v>
+      </c>
+      <c r="J8" t="s">
+        <v>205</v>
+      </c>
+      <c r="K8" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>149</v>
+      </c>
+      <c r="B9" t="s">
+        <v>132</v>
+      </c>
+      <c r="C9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D9" t="s">
+        <v>160</v>
+      </c>
+      <c r="E9" t="s">
+        <v>147</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H9">
+        <v>1.05</v>
+      </c>
+      <c r="I9" t="s">
+        <v>204</v>
+      </c>
+      <c r="J9" t="s">
+        <v>205</v>
+      </c>
+      <c r="K9" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C10" t="s">
+        <v>159</v>
+      </c>
+      <c r="D10" t="s">
+        <v>160</v>
+      </c>
+      <c r="E10" t="s">
+        <v>147</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="H10">
+        <v>1.08</v>
+      </c>
+      <c r="I10" t="s">
+        <v>204</v>
+      </c>
+      <c r="J10" t="s">
+        <v>205</v>
+      </c>
+      <c r="K10" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C11" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="E11" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11">
+        <v>0.85</v>
+      </c>
+      <c r="G11">
+        <v>0.85</v>
+      </c>
+      <c r="H11">
+        <v>0.95</v>
+      </c>
+      <c r="I11" t="s">
+        <v>211</v>
+      </c>
+      <c r="J11" t="s">
+        <v>205</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12">
+        <v>0.9</v>
+      </c>
+      <c r="G12">
+        <v>0.95</v>
+      </c>
+      <c r="H12">
+        <v>0.98</v>
+      </c>
+      <c r="I12" t="s">
+        <v>213</v>
+      </c>
+      <c r="J12" t="s">
+        <v>205</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D13" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="H13">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="I13" t="s">
+        <v>215</v>
+      </c>
+      <c r="J13" t="s">
+        <v>205</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="D3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E3">
-        <v>0.8</v>
-      </c>
-      <c r="F3">
-        <v>1.08</v>
-      </c>
-      <c r="G3">
-        <v>1.1100000000000001</v>
-      </c>
-      <c r="H3" t="s">
-        <v>130</v>
-      </c>
-      <c r="I3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" t="s">
-        <v>131</v>
-      </c>
-      <c r="C4" t="s">
-        <v>132</v>
-      </c>
-      <c r="D4" t="s">
-        <v>72</v>
-      </c>
-      <c r="E4">
-        <v>0.8</v>
-      </c>
-      <c r="F4">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="G4">
-        <v>1.2</v>
-      </c>
-      <c r="H4" t="s">
-        <v>130</v>
-      </c>
-      <c r="I4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>133</v>
-      </c>
-      <c r="B5" t="s">
-        <v>134</v>
-      </c>
-      <c r="C5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="E14" t="s">
         <v>76</v>
       </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="G5">
-        <v>1.05</v>
-      </c>
-      <c r="H5" t="s">
-        <v>130</v>
-      </c>
-      <c r="I5" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>135</v>
-      </c>
-      <c r="B6" t="s">
-        <v>136</v>
-      </c>
-      <c r="C6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="F6">
-        <v>1.08</v>
-      </c>
-      <c r="G6">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="H6" t="s">
-        <v>137</v>
-      </c>
-      <c r="I6" t="s">
-        <v>124</v>
-      </c>
-      <c r="J6" t="s">
-        <v>138</v>
+      <c r="F14">
+        <v>0.9</v>
+      </c>
+      <c r="G14">
+        <v>0.95</v>
+      </c>
+      <c r="H14">
+        <v>0.98</v>
+      </c>
+      <c r="I14" t="s">
+        <v>213</v>
+      </c>
+      <c r="J14" t="s">
+        <v>205</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -2980,7 +3357,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41DDFEBE-0F4B-4A30-8443-0DC0960E2CAF}">
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -2991,17 +3368,18 @@
     <col min="6" max="6" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="22.42578125" customWidth="1"/>
+    <col min="11" max="11" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -3014,44 +3392,50 @@
       <c r="D1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="5" t="s">
         <v>37</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>38</v>
       </c>
       <c r="I1" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="P1" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -3064,41 +3448,47 @@
       <c r="D2">
         <v>125.4</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="6" t="s">
         <v>49</v>
       </c>
       <c r="H2" t="s">
         <v>50</v>
       </c>
       <c r="I2" t="s">
+        <v>218</v>
+      </c>
+      <c r="J2">
+        <v>5</v>
+      </c>
+      <c r="K2" t="s">
         <v>71</v>
       </c>
-      <c r="J2" t="s">
+      <c r="L2" t="s">
         <v>72</v>
       </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
         <v>51</v>
       </c>
-      <c r="L2" t="s">
+      <c r="N2" t="s">
         <v>51</v>
       </c>
-      <c r="M2" t="s">
+      <c r="O2" t="s">
         <v>49</v>
       </c>
-      <c r="N2" t="s">
+      <c r="P2" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="O2" s="1">
+      <c r="Q2" s="1">
         <v>46023</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -3111,88 +3501,578 @@
       <c r="D3">
         <v>89.7</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="6" t="s">
         <v>49</v>
       </c>
       <c r="H3" t="s">
         <v>57</v>
       </c>
       <c r="I3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J3">
+        <v>8</v>
+      </c>
+      <c r="K3" t="s">
         <v>71</v>
       </c>
-      <c r="J3" t="s">
+      <c r="L3" t="s">
         <v>76</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
         <v>51</v>
       </c>
-      <c r="L3" t="s">
+      <c r="N3" t="s">
         <v>51</v>
       </c>
-      <c r="M3" t="s">
+      <c r="O3" t="s">
         <v>49</v>
       </c>
-      <c r="N3" t="s">
+      <c r="P3" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="O3" s="1">
+      <c r="Q3" s="1">
         <v>46023</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D4">
         <v>150</v>
       </c>
+      <c r="E4" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="H4" t="s">
+        <v>159</v>
+      </c>
+      <c r="I4" t="s">
+        <v>220</v>
+      </c>
+      <c r="J4">
+        <v>9</v>
+      </c>
+      <c r="K4" t="s">
+        <v>160</v>
+      </c>
+      <c r="L4" t="s">
+        <v>147</v>
+      </c>
+      <c r="M4" t="s">
+        <v>161</v>
+      </c>
+      <c r="N4" t="s">
+        <v>51</v>
+      </c>
+      <c r="O4" t="s">
+        <v>132</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>45292</v>
+      </c>
+      <c r="R4" t="s">
+        <v>163</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EECD6AE4-F479-47F2-A7D9-6780452D29FE}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="A2:N11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="1">
+        <v>46127</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>10</v>
+      </c>
+      <c r="I3">
+        <v>1.85</v>
+      </c>
+      <c r="J3">
+        <v>1.28</v>
+      </c>
+      <c r="K3">
+        <v>0.05</v>
+      </c>
+      <c r="L3">
+        <v>18.2</v>
+      </c>
+      <c r="M3">
+        <v>6.4</v>
+      </c>
+      <c r="N3" s="9">
+        <f>I3*J3*(H3-G3)*(1-K3)*0.1</f>
+        <v>2.2496000000000005</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
       <c r="E4" t="s">
-        <v>150</v>
-      </c>
-      <c r="F4" t="s">
-        <v>159</v>
-      </c>
-      <c r="G4" t="s">
-        <v>133</v>
-      </c>
-      <c r="H4" t="s">
-        <v>160</v>
-      </c>
-      <c r="I4" t="s">
-        <v>161</v>
-      </c>
-      <c r="J4" t="s">
-        <v>148</v>
-      </c>
-      <c r="K4" t="s">
-        <v>162</v>
-      </c>
-      <c r="L4" t="s">
-        <v>51</v>
-      </c>
-      <c r="M4" t="s">
-        <v>133</v>
-      </c>
-      <c r="N4" t="s">
-        <v>163</v>
-      </c>
-      <c r="O4" s="1">
-        <v>45292</v>
-      </c>
-      <c r="P4" t="s">
-        <v>164</v>
+        <v>22</v>
+      </c>
+      <c r="F4" s="1">
+        <v>46127</v>
+      </c>
+      <c r="G4">
+        <v>10</v>
+      </c>
+      <c r="H4">
+        <v>30</v>
+      </c>
+      <c r="I4">
+        <v>1.22</v>
+      </c>
+      <c r="J4">
+        <v>1.36</v>
+      </c>
+      <c r="K4">
+        <v>0.08</v>
+      </c>
+      <c r="L4">
+        <v>20.5</v>
+      </c>
+      <c r="M4">
+        <v>6.3</v>
+      </c>
+      <c r="N4" s="9">
+        <f t="shared" ref="N4:N11" si="0">I4*J4*(H4-G4)*(1-K4)*0.1</f>
+        <v>3.0529280000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="1">
+        <v>46129</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>10</v>
+      </c>
+      <c r="I5">
+        <v>2.1</v>
+      </c>
+      <c r="J5">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="K5">
+        <v>0.02</v>
+      </c>
+      <c r="L5">
+        <v>22</v>
+      </c>
+      <c r="M5">
+        <v>6.8</v>
+      </c>
+      <c r="N5" s="9">
+        <f t="shared" si="0"/>
+        <v>2.2843800000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s">
+        <v>168</v>
+      </c>
+      <c r="E6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F6" s="1">
+        <v>45181</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="I6">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="J6">
+        <v>1.48</v>
+      </c>
+      <c r="K6">
+        <v>0.06</v>
+      </c>
+      <c r="L6">
+        <v>17.5</v>
+      </c>
+      <c r="M6">
+        <v>5.9</v>
+      </c>
+      <c r="N6" s="9">
+        <f t="shared" si="0"/>
+        <v>1.5303200000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B7" t="s">
+        <v>141</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E7" t="s">
+        <v>192</v>
+      </c>
+      <c r="F7" s="1">
+        <v>45181</v>
+      </c>
+      <c r="G7">
+        <v>10</v>
+      </c>
+      <c r="H7">
+        <v>30</v>
+      </c>
+      <c r="I7">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="J7">
+        <v>1.52</v>
+      </c>
+      <c r="K7">
+        <v>0.08</v>
+      </c>
+      <c r="L7">
+        <v>19</v>
+      </c>
+      <c r="M7">
+        <v>6</v>
+      </c>
+      <c r="N7" s="9">
+        <f t="shared" si="0"/>
+        <v>1.5382400000000003</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" t="s">
+        <v>169</v>
+      </c>
+      <c r="E8" t="s">
+        <v>192</v>
+      </c>
+      <c r="F8" s="1">
+        <v>45182</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>10</v>
+      </c>
+      <c r="I8">
+        <v>1.25</v>
+      </c>
+      <c r="J8">
+        <v>1.46</v>
+      </c>
+      <c r="K8">
+        <v>0.05</v>
+      </c>
+      <c r="L8">
+        <v>18.8</v>
+      </c>
+      <c r="M8">
+        <v>5.8</v>
+      </c>
+      <c r="N8" s="9">
+        <f t="shared" si="0"/>
+        <v>1.7337499999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>194</v>
+      </c>
+      <c r="B9" t="s">
+        <v>141</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
+        <v>169</v>
+      </c>
+      <c r="E9" t="s">
+        <v>192</v>
+      </c>
+      <c r="F9" s="1">
+        <v>45182</v>
+      </c>
+      <c r="G9">
+        <v>10</v>
+      </c>
+      <c r="H9">
+        <v>30</v>
+      </c>
+      <c r="I9">
+        <v>0.6</v>
+      </c>
+      <c r="J9">
+        <v>1.5</v>
+      </c>
+      <c r="K9">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L9">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="M9">
+        <v>5.9</v>
+      </c>
+      <c r="N9" s="9">
+        <f t="shared" si="0"/>
+        <v>1.6739999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>195</v>
+      </c>
+      <c r="B10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" t="s">
+        <v>170</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="1">
+        <v>46132</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>10</v>
+      </c>
+      <c r="I10">
+        <v>1.65</v>
+      </c>
+      <c r="J10">
+        <v>1.42</v>
+      </c>
+      <c r="K10">
+        <v>0.04</v>
+      </c>
+      <c r="L10">
+        <v>21</v>
+      </c>
+      <c r="M10">
+        <v>6.2</v>
+      </c>
+      <c r="N10" s="9">
+        <f t="shared" si="0"/>
+        <v>2.2492800000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>196</v>
+      </c>
+      <c r="B11" t="s">
+        <v>141</v>
+      </c>
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" t="s">
+        <v>170</v>
+      </c>
+      <c r="E11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="1">
+        <v>46132</v>
+      </c>
+      <c r="G11">
+        <v>10</v>
+      </c>
+      <c r="H11">
+        <v>30</v>
+      </c>
+      <c r="I11">
+        <v>0.95</v>
+      </c>
+      <c r="J11">
+        <v>1.47</v>
+      </c>
+      <c r="K11">
+        <v>0.06</v>
+      </c>
+      <c r="L11">
+        <v>22.3</v>
+      </c>
+      <c r="M11">
+        <v>6.1</v>
+      </c>
+      <c r="N11" s="9">
+        <f t="shared" si="0"/>
+        <v>2.6254199999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expand README with detailed SOC accounting logic, demo project examples, and PDF generation instructions.
</commit_message>
<xml_diff>
--- a/data/my_project/raw/my_data.xlsx
+++ b/data/my_project/raw/my_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tboll\DELL_local_code\CarbonIQ\agricultural-land-management\data\my_project\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560D2A48-5A4E-404C-90A8-AA9FA17F7EDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D74D12-5E45-4B76-9ADC-A092EFC64561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="750" yWindow="1245" windowWidth="26400" windowHeight="15645" firstSheet="1" activeTab="7" xr2:uid="{9B51F04F-7C9B-484C-9CA7-D1EDE120DFB6}"/>
+    <workbookView xWindow="750" yWindow="1245" windowWidth="26400" windowHeight="15645" xr2:uid="{9B51F04F-7C9B-484C-9CA7-D1EDE120DFB6}"/>
   </bookViews>
   <sheets>
     <sheet name="projects" sheetId="5" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="225">
   <si>
     <t>sample_id</t>
   </si>
@@ -713,6 +713,12 @@
   </si>
   <si>
     <t>stock_tC_ha</t>
+  </si>
+  <si>
+    <t>ipcc_stock</t>
+  </si>
+  <si>
+    <t>SOCSAMP_001_0004</t>
   </si>
 </sst>
 </file>
@@ -2246,7 +2252,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2CAEEC4-1B47-4A4C-AFB2-5EDCA6AA40D8}">
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
@@ -2499,66 +2505,63 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>174</v>
+        <v>224</v>
       </c>
       <c r="B5" t="s">
-        <v>141</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>168</v>
+        <v>27</v>
       </c>
       <c r="E5" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="F5" s="1">
-        <v>45181</v>
+        <v>46129</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H5">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="I5">
-        <v>1.1000000000000001</v>
+        <v>1.85</v>
       </c>
       <c r="J5">
-        <v>1.48</v>
+        <v>1.2</v>
       </c>
       <c r="K5">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="L5">
-        <v>17.5</v>
+        <v>24</v>
       </c>
       <c r="M5">
-        <v>5.9</v>
+        <v>6.7</v>
       </c>
       <c r="N5" t="s">
-        <v>193</v>
+        <v>28</v>
       </c>
       <c r="O5" t="s">
         <v>24</v>
       </c>
       <c r="P5">
-        <v>-31.5</v>
+        <v>34.127000000000002</v>
       </c>
       <c r="Q5">
-        <v>151.5</v>
+        <v>-118.355</v>
       </c>
       <c r="R5" t="s">
         <v>25</v>
       </c>
-      <c r="S5" t="s">
-        <v>197</v>
-      </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B6" t="s">
         <v>141</v>
@@ -2576,25 +2579,25 @@
         <v>45181</v>
       </c>
       <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
         <v>10</v>
       </c>
-      <c r="H6">
-        <v>30</v>
-      </c>
       <c r="I6">
-        <v>0.55000000000000004</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="J6">
-        <v>1.52</v>
+        <v>1.48</v>
       </c>
       <c r="K6">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="L6">
-        <v>19</v>
+        <v>17.5</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="N6" t="s">
         <v>193</v>
@@ -2612,12 +2615,12 @@
         <v>25</v>
       </c>
       <c r="S6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B7" t="s">
         <v>141</v>
@@ -2626,34 +2629,34 @@
         <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E7" t="s">
         <v>192</v>
       </c>
       <c r="F7" s="1">
-        <v>45182</v>
+        <v>45181</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H7">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="I7">
-        <v>1.25</v>
+        <v>0.65</v>
       </c>
       <c r="J7">
-        <v>1.46</v>
+        <v>1.52</v>
       </c>
       <c r="K7">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="L7">
-        <v>18.8</v>
+        <v>19</v>
       </c>
       <c r="M7">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="N7" t="s">
         <v>193</v>
@@ -2662,21 +2665,21 @@
         <v>24</v>
       </c>
       <c r="P7">
-        <v>-31.502500000000001</v>
+        <v>-31.5</v>
       </c>
       <c r="Q7">
-        <v>151.50299999999999</v>
+        <v>151.5</v>
       </c>
       <c r="R7" t="s">
         <v>25</v>
       </c>
       <c r="S7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>194</v>
+        <v>176</v>
       </c>
       <c r="B8" t="s">
         <v>141</v>
@@ -2694,25 +2697,25 @@
         <v>45182</v>
       </c>
       <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
         <v>10</v>
       </c>
-      <c r="H8">
-        <v>30</v>
-      </c>
       <c r="I8">
-        <v>0.6</v>
+        <v>1.25</v>
       </c>
       <c r="J8">
-        <v>1.5</v>
+        <v>1.46</v>
       </c>
       <c r="K8">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="L8">
-        <v>20.100000000000001</v>
+        <v>18.8</v>
       </c>
       <c r="M8">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="N8" t="s">
         <v>193</v>
@@ -2730,12 +2733,12 @@
         <v>25</v>
       </c>
       <c r="S8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B9" t="s">
         <v>141</v>
@@ -2744,34 +2747,34 @@
         <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E9" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="F9" s="1">
-        <v>46132</v>
+        <v>45182</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H9">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="I9">
-        <v>1.65</v>
+        <v>0.8</v>
       </c>
       <c r="J9">
-        <v>1.42</v>
+        <v>1.5</v>
       </c>
       <c r="K9">
-        <v>0.04</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="L9">
-        <v>21</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="M9">
-        <v>6.2</v>
+        <v>5.9</v>
       </c>
       <c r="N9" t="s">
         <v>193</v>
@@ -2780,21 +2783,21 @@
         <v>24</v>
       </c>
       <c r="P9">
-        <v>-31.498000000000001</v>
+        <v>-31.502500000000001</v>
       </c>
       <c r="Q9">
-        <v>151.49700000000001</v>
+        <v>151.50299999999999</v>
       </c>
       <c r="R9" t="s">
         <v>25</v>
       </c>
       <c r="S9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B10" t="s">
         <v>141</v>
@@ -2812,25 +2815,25 @@
         <v>46132</v>
       </c>
       <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
         <v>10</v>
       </c>
-      <c r="H10">
-        <v>30</v>
-      </c>
       <c r="I10">
-        <v>0.95</v>
+        <v>1.65</v>
       </c>
       <c r="J10">
-        <v>1.47</v>
+        <v>1.42</v>
       </c>
       <c r="K10">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="L10">
-        <v>22.3</v>
+        <v>21</v>
       </c>
       <c r="M10">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="N10" t="s">
         <v>193</v>
@@ -2848,6 +2851,65 @@
         <v>25</v>
       </c>
       <c r="S10" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>196</v>
+      </c>
+      <c r="B11" t="s">
+        <v>141</v>
+      </c>
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" t="s">
+        <v>170</v>
+      </c>
+      <c r="E11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="1">
+        <v>46132</v>
+      </c>
+      <c r="G11">
+        <v>10</v>
+      </c>
+      <c r="H11">
+        <v>30</v>
+      </c>
+      <c r="I11">
+        <v>0.95</v>
+      </c>
+      <c r="J11">
+        <v>1.47</v>
+      </c>
+      <c r="K11">
+        <v>0.06</v>
+      </c>
+      <c r="L11">
+        <v>22.3</v>
+      </c>
+      <c r="M11">
+        <v>6.1</v>
+      </c>
+      <c r="N11" t="s">
+        <v>193</v>
+      </c>
+      <c r="O11" t="s">
+        <v>24</v>
+      </c>
+      <c r="P11">
+        <v>-31.498000000000001</v>
+      </c>
+      <c r="Q11">
+        <v>151.49700000000001</v>
+      </c>
+      <c r="R11" t="s">
+        <v>25</v>
+      </c>
+      <c r="S11" t="s">
         <v>202</v>
       </c>
     </row>
@@ -3607,7 +3669,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A2:N11"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
@@ -3618,7 +3680,7 @@
     <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="24.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="17.28515625" bestFit="1" customWidth="1"/>
@@ -3626,453 +3688,1015 @@
     <col min="14" max="14" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="D2" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2">
+        <f>SUMIF($D$11:$D$21,$D2,N$11:N$21)</f>
+        <v>53.025280000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
+        <v>27</v>
+      </c>
+      <c r="N3">
+        <f t="shared" ref="N3:N6" si="0">SUMIF($D$11:$D$21,$D3,N$11:N$21)</f>
+        <v>63.691800000000008</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>168</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="0"/>
+        <v>33.482399999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>169</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="0"/>
+        <v>39.657499999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>170</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="0"/>
+        <v>48.746999999999993</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N11" s="2" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>171</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B12" t="s">
         <v>19</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C12" t="s">
         <v>20</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D12" t="s">
         <v>21</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E12" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F12" s="1">
         <v>46127</v>
       </c>
-      <c r="G3">
+      <c r="G12">
         <v>0</v>
       </c>
-      <c r="H3">
+      <c r="H12">
         <v>10</v>
       </c>
-      <c r="I3">
+      <c r="I12">
         <v>1.85</v>
       </c>
-      <c r="J3">
+      <c r="J12">
         <v>1.28</v>
       </c>
-      <c r="K3">
+      <c r="K12">
         <v>0.05</v>
       </c>
-      <c r="L3">
+      <c r="L12">
         <v>18.2</v>
       </c>
-      <c r="M3">
+      <c r="M12">
         <v>6.4</v>
       </c>
-      <c r="N3" s="9">
-        <f>I3*J3*(H3-G3)*(1-K3)*0.1</f>
-        <v>2.2496000000000005</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="N12" s="9">
+        <f>I12*J12*(H12-G12)*(1-K12)</f>
+        <v>22.496000000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>172</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B13" t="s">
         <v>19</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C13" t="s">
         <v>20</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D13" t="s">
         <v>21</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E13" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F13" s="1">
         <v>46127</v>
       </c>
-      <c r="G4">
+      <c r="G13">
         <v>10</v>
       </c>
-      <c r="H4">
+      <c r="H13">
         <v>30</v>
       </c>
-      <c r="I4">
+      <c r="I13">
         <v>1.22</v>
       </c>
-      <c r="J4">
+      <c r="J13">
         <v>1.36</v>
       </c>
-      <c r="K4">
+      <c r="K13">
         <v>0.08</v>
       </c>
-      <c r="L4">
+      <c r="L13">
         <v>20.5</v>
       </c>
-      <c r="M4">
+      <c r="M13">
         <v>6.3</v>
       </c>
-      <c r="N4" s="9">
-        <f t="shared" ref="N4:N11" si="0">I4*J4*(H4-G4)*(1-K4)*0.1</f>
-        <v>3.0529280000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="N13" s="9">
+        <f t="shared" ref="N13:N21" si="1">I13*J13*(H13-G13)*(1-K13)</f>
+        <v>30.52928</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>173</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B14" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C14" t="s">
         <v>26</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D14" t="s">
         <v>27</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E14" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F14" s="1">
         <v>46129</v>
       </c>
-      <c r="G5">
+      <c r="G14">
         <v>0</v>
       </c>
-      <c r="H5">
+      <c r="H14">
         <v>10</v>
       </c>
-      <c r="I5">
+      <c r="I14">
         <v>2.1</v>
       </c>
-      <c r="J5">
+      <c r="J14">
         <v>1.1100000000000001</v>
       </c>
-      <c r="K5">
+      <c r="K14">
         <v>0.02</v>
       </c>
-      <c r="L5">
+      <c r="L14">
         <v>22</v>
       </c>
-      <c r="M5">
+      <c r="M14">
         <v>6.8</v>
       </c>
-      <c r="N5" s="9">
-        <f t="shared" si="0"/>
-        <v>2.2843800000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="N14" s="9">
+        <f t="shared" si="1"/>
+        <v>22.843800000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>224</v>
+      </c>
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="1">
+        <v>46129</v>
+      </c>
+      <c r="G15">
+        <v>10</v>
+      </c>
+      <c r="H15">
+        <v>30</v>
+      </c>
+      <c r="I15">
+        <v>1.85</v>
+      </c>
+      <c r="J15">
+        <v>1.2</v>
+      </c>
+      <c r="K15">
+        <v>0.08</v>
+      </c>
+      <c r="L15">
+        <v>24</v>
+      </c>
+      <c r="M15">
+        <v>6.7</v>
+      </c>
+      <c r="N15" s="9">
+        <f t="shared" si="1"/>
+        <v>40.848000000000006</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>174</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B16" t="s">
         <v>141</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C16" t="s">
         <v>20</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D16" t="s">
         <v>168</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E16" t="s">
         <v>192</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F16" s="1">
         <v>45181</v>
       </c>
-      <c r="G6">
+      <c r="G16">
         <v>0</v>
       </c>
-      <c r="H6">
+      <c r="H16">
         <v>10</v>
       </c>
-      <c r="I6">
+      <c r="I16">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J6">
+      <c r="J16">
         <v>1.48</v>
       </c>
-      <c r="K6">
+      <c r="K16">
         <v>0.06</v>
       </c>
-      <c r="L6">
+      <c r="L16">
         <v>17.5</v>
       </c>
-      <c r="M6">
+      <c r="M16">
         <v>5.9</v>
       </c>
-      <c r="N6" s="9">
-        <f t="shared" si="0"/>
-        <v>1.5303200000000001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="N16" s="9">
+        <f t="shared" si="1"/>
+        <v>15.3032</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>175</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B17" t="s">
         <v>141</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C17" t="s">
         <v>20</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D17" t="s">
         <v>168</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E17" t="s">
         <v>192</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F17" s="1">
         <v>45181</v>
       </c>
-      <c r="G7">
+      <c r="G17">
         <v>10</v>
       </c>
-      <c r="H7">
+      <c r="H17">
         <v>30</v>
       </c>
-      <c r="I7">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="J7">
+      <c r="I17">
+        <v>0.65</v>
+      </c>
+      <c r="J17">
         <v>1.52</v>
       </c>
-      <c r="K7">
+      <c r="K17">
         <v>0.08</v>
       </c>
-      <c r="L7">
+      <c r="L17">
         <v>19</v>
       </c>
-      <c r="M7">
+      <c r="M17">
         <v>6</v>
       </c>
-      <c r="N7" s="9">
-        <f t="shared" si="0"/>
-        <v>1.5382400000000003</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="N17" s="9">
+        <f t="shared" si="1"/>
+        <v>18.179200000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>176</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B18" t="s">
         <v>141</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C18" t="s">
         <v>20</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D18" t="s">
         <v>169</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E18" t="s">
         <v>192</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F18" s="1">
         <v>45182</v>
       </c>
-      <c r="G8">
+      <c r="G18">
         <v>0</v>
       </c>
-      <c r="H8">
+      <c r="H18">
         <v>10</v>
       </c>
-      <c r="I8">
+      <c r="I18">
         <v>1.25</v>
       </c>
-      <c r="J8">
+      <c r="J18">
         <v>1.46</v>
       </c>
-      <c r="K8">
+      <c r="K18">
         <v>0.05</v>
       </c>
-      <c r="L8">
+      <c r="L18">
         <v>18.8</v>
       </c>
-      <c r="M8">
+      <c r="M18">
         <v>5.8</v>
       </c>
-      <c r="N8" s="9">
-        <f t="shared" si="0"/>
-        <v>1.7337499999999999</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="N18" s="9">
+        <f t="shared" si="1"/>
+        <v>17.337499999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>194</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B19" t="s">
         <v>141</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C19" t="s">
         <v>20</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D19" t="s">
         <v>169</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E19" t="s">
         <v>192</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F19" s="1">
         <v>45182</v>
       </c>
-      <c r="G9">
+      <c r="G19">
         <v>10</v>
       </c>
-      <c r="H9">
+      <c r="H19">
         <v>30</v>
       </c>
-      <c r="I9">
-        <v>0.6</v>
-      </c>
-      <c r="J9">
+      <c r="I19">
+        <v>0.8</v>
+      </c>
+      <c r="J19">
         <v>1.5</v>
       </c>
-      <c r="K9">
+      <c r="K19">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="L9">
+      <c r="L19">
         <v>20.100000000000001</v>
       </c>
-      <c r="M9">
+      <c r="M19">
         <v>5.9</v>
       </c>
-      <c r="N9" s="9">
-        <f t="shared" si="0"/>
-        <v>1.6739999999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="N19" s="9">
+        <f t="shared" si="1"/>
+        <v>22.32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>195</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B20" t="s">
         <v>141</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C20" t="s">
         <v>20</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D20" t="s">
         <v>170</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E20" t="s">
         <v>22</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F20" s="1">
         <v>46132</v>
       </c>
-      <c r="G10">
+      <c r="G20">
         <v>0</v>
       </c>
-      <c r="H10">
+      <c r="H20">
         <v>10</v>
       </c>
-      <c r="I10">
+      <c r="I20">
         <v>1.65</v>
       </c>
-      <c r="J10">
+      <c r="J20">
         <v>1.42</v>
       </c>
-      <c r="K10">
+      <c r="K20">
         <v>0.04</v>
       </c>
-      <c r="L10">
+      <c r="L20">
         <v>21</v>
       </c>
-      <c r="M10">
+      <c r="M20">
         <v>6.2</v>
       </c>
-      <c r="N10" s="9">
-        <f t="shared" si="0"/>
-        <v>2.2492800000000002</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="N20" s="9">
+        <f t="shared" si="1"/>
+        <v>22.492799999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>196</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B21" t="s">
         <v>141</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C21" t="s">
         <v>20</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D21" t="s">
         <v>170</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E21" t="s">
         <v>22</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F21" s="1">
         <v>46132</v>
       </c>
-      <c r="G11">
+      <c r="G21">
         <v>10</v>
       </c>
-      <c r="H11">
+      <c r="H21">
         <v>30</v>
       </c>
-      <c r="I11">
+      <c r="I21">
         <v>0.95</v>
       </c>
-      <c r="J11">
+      <c r="J21">
         <v>1.47</v>
       </c>
-      <c r="K11">
+      <c r="K21">
         <v>0.06</v>
       </c>
-      <c r="L11">
+      <c r="L21">
         <v>22.3</v>
       </c>
-      <c r="M11">
+      <c r="M21">
         <v>6.1</v>
       </c>
-      <c r="N11" s="9">
-        <f t="shared" si="0"/>
-        <v>2.6254199999999996</v>
+      <c r="N21" s="9">
+        <f t="shared" si="1"/>
+        <v>26.254199999999994</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="K25" s="2"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>203</v>
+      </c>
+      <c r="B26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" t="s">
+        <v>71</v>
+      </c>
+      <c r="E26" t="s">
+        <v>76</v>
+      </c>
+      <c r="F26">
+        <v>0.8</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26">
+        <v>38</v>
+      </c>
+      <c r="J26">
+        <f>I26*F26*G26*H26</f>
+        <v>30.400000000000002</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>203</v>
+      </c>
+      <c r="B27" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27" t="s">
+        <v>50</v>
+      </c>
+      <c r="D27" t="s">
+        <v>71</v>
+      </c>
+      <c r="E27" t="s">
+        <v>72</v>
+      </c>
+      <c r="F27">
+        <v>0.8</v>
+      </c>
+      <c r="G27">
+        <v>1.08</v>
+      </c>
+      <c r="H27">
+        <v>1.1100000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>203</v>
+      </c>
+      <c r="B28" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" t="s">
+        <v>130</v>
+      </c>
+      <c r="D28" t="s">
+        <v>131</v>
+      </c>
+      <c r="E28" t="s">
+        <v>72</v>
+      </c>
+      <c r="F28">
+        <v>0.8</v>
+      </c>
+      <c r="G28">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="H28">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>203</v>
+      </c>
+      <c r="B29" t="s">
+        <v>132</v>
+      </c>
+      <c r="C29" t="s">
+        <v>133</v>
+      </c>
+      <c r="D29" t="s">
+        <v>71</v>
+      </c>
+      <c r="E29" t="s">
+        <v>76</v>
+      </c>
+      <c r="F29">
+        <v>1</v>
+      </c>
+      <c r="G29">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H29">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>203</v>
+      </c>
+      <c r="B30" t="s">
+        <v>134</v>
+      </c>
+      <c r="C30" t="s">
+        <v>135</v>
+      </c>
+      <c r="D30" t="s">
+        <v>71</v>
+      </c>
+      <c r="E30" t="s">
+        <v>72</v>
+      </c>
+      <c r="F30">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="G30">
+        <v>1.08</v>
+      </c>
+      <c r="H30">
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="D31" t="s">
+        <v>160</v>
+      </c>
+      <c r="E31" t="s">
+        <v>147</v>
+      </c>
+      <c r="F31">
+        <v>1</v>
+      </c>
+      <c r="G31">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="H31">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>149</v>
+      </c>
+      <c r="B32" t="s">
+        <v>132</v>
+      </c>
+      <c r="C32" t="s">
+        <v>162</v>
+      </c>
+      <c r="D32" t="s">
+        <v>160</v>
+      </c>
+      <c r="E32" t="s">
+        <v>147</v>
+      </c>
+      <c r="F32">
+        <v>0.95</v>
+      </c>
+      <c r="G32">
+        <v>0.95</v>
+      </c>
+      <c r="H32">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>149</v>
+      </c>
+      <c r="B33" t="s">
+        <v>132</v>
+      </c>
+      <c r="C33" t="s">
+        <v>133</v>
+      </c>
+      <c r="D33" t="s">
+        <v>160</v>
+      </c>
+      <c r="E33" t="s">
+        <v>147</v>
+      </c>
+      <c r="F33">
+        <v>1</v>
+      </c>
+      <c r="G33">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H33">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>149</v>
+      </c>
+      <c r="B34" t="s">
+        <v>132</v>
+      </c>
+      <c r="C34" t="s">
+        <v>159</v>
+      </c>
+      <c r="D34" t="s">
+        <v>160</v>
+      </c>
+      <c r="E34" t="s">
+        <v>147</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+      <c r="G34">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="H34">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="E35" t="s">
+        <v>76</v>
+      </c>
+      <c r="F35">
+        <v>0.85</v>
+      </c>
+      <c r="G35">
+        <v>0.85</v>
+      </c>
+      <c r="H35">
+        <v>0.95</v>
+      </c>
+      <c r="K35" s="8"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E36" t="s">
+        <v>76</v>
+      </c>
+      <c r="F36">
+        <v>0.9</v>
+      </c>
+      <c r="G36">
+        <v>0.95</v>
+      </c>
+      <c r="H36">
+        <v>0.98</v>
+      </c>
+      <c r="K36" s="8"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="F37">
+        <v>1</v>
+      </c>
+      <c r="G37">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="H37">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="K37" s="8"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E38" t="s">
+        <v>76</v>
+      </c>
+      <c r="F38">
+        <v>0.9</v>
+      </c>
+      <c r="G38">
+        <v>0.95</v>
+      </c>
+      <c r="H38">
+        <v>0.98</v>
+      </c>
+      <c r="K38" s="8"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>48</v>
+      </c>
+      <c r="B42" t="s">
+        <v>70</v>
+      </c>
+      <c r="C42">
+        <v>30</v>
+      </c>
+      <c r="D42">
+        <v>38</v>
+      </c>
+      <c r="E42" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>48</v>
+      </c>
+      <c r="B43" t="s">
+        <v>75</v>
+      </c>
+      <c r="C43">
+        <v>30</v>
+      </c>
+      <c r="D43">
+        <v>46</v>
+      </c>
+      <c r="E43" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>125</v>
+      </c>
+      <c r="B44" t="s">
+        <v>70</v>
+      </c>
+      <c r="C44">
+        <v>30</v>
+      </c>
+      <c r="D44">
+        <v>62</v>
+      </c>
+      <c r="E44" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>149</v>
+      </c>
+      <c r="B45" t="s">
+        <v>158</v>
+      </c>
+      <c r="C45">
+        <v>30</v>
+      </c>
+      <c r="D45">
+        <v>48</v>
+      </c>
+      <c r="E45" t="s">
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>